<commit_message>
fixed to product reviews
</commit_message>
<xml_diff>
--- a/catalog.xlsx
+++ b/catalog.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R71"/>
+  <dimension ref="A1:R92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -571,7 +571,6 @@
       <c r="N2" t="n">
         <v>1</v>
       </c>
-      <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr">
         <is>
           <t>CJKT3151335</t>
@@ -651,7 +650,6 @@
       <c r="N3" t="n">
         <v>1</v>
       </c>
-      <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr">
         <is>
           <t>CJTZ3113454</t>
@@ -731,7 +729,6 @@
       <c r="N4" t="n">
         <v>1</v>
       </c>
-      <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr">
         <is>
           <t>CJMY3090389</t>
@@ -811,7 +808,6 @@
       <c r="N5" t="n">
         <v>1</v>
       </c>
-      <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr">
         <is>
           <t>CJTZ3091878</t>
@@ -891,7 +887,6 @@
       <c r="N6" t="n">
         <v>1</v>
       </c>
-      <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr">
         <is>
           <t>CJLY3083517</t>
@@ -971,7 +966,6 @@
       <c r="N7" t="n">
         <v>1</v>
       </c>
-      <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr">
         <is>
           <t>CJWO3078837</t>
@@ -1051,7 +1045,6 @@
       <c r="N8" t="n">
         <v>1</v>
       </c>
-      <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr">
         <is>
           <t>CJTZ3077271</t>
@@ -1131,7 +1124,6 @@
       <c r="N9" t="n">
         <v>1</v>
       </c>
-      <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr">
         <is>
           <t>CJTZ3071585</t>
@@ -1211,7 +1203,6 @@
       <c r="N10" t="n">
         <v>1</v>
       </c>
-      <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr">
         <is>
           <t>CJWL3066864</t>
@@ -1291,7 +1282,6 @@
       <c r="N11" t="n">
         <v>1</v>
       </c>
-      <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr">
         <is>
           <t>CJTZ3067953</t>
@@ -1371,7 +1361,6 @@
       <c r="N12" t="n">
         <v>1</v>
       </c>
-      <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr">
         <is>
           <t>CJKT3059304</t>
@@ -1451,7 +1440,6 @@
       <c r="N13" t="n">
         <v>1</v>
       </c>
-      <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr">
         <is>
           <t>CJTZ3061309</t>
@@ -1531,7 +1519,6 @@
       <c r="N14" t="n">
         <v>1</v>
       </c>
-      <c r="O14" t="inlineStr"/>
       <c r="P14" t="inlineStr">
         <is>
           <t>CJTZ3057756</t>
@@ -1611,7 +1598,6 @@
       <c r="N15" t="n">
         <v>1</v>
       </c>
-      <c r="O15" t="inlineStr"/>
       <c r="P15" t="inlineStr">
         <is>
           <t>CJQB3057928</t>
@@ -1691,7 +1677,6 @@
       <c r="N16" t="n">
         <v>1</v>
       </c>
-      <c r="O16" t="inlineStr"/>
       <c r="P16" t="inlineStr">
         <is>
           <t>CJTZ3055387</t>
@@ -1771,7 +1756,6 @@
       <c r="N17" t="n">
         <v>1</v>
       </c>
-      <c r="O17" t="inlineStr"/>
       <c r="P17" t="inlineStr">
         <is>
           <t>CJLT3048464</t>
@@ -1851,7 +1835,6 @@
       <c r="N18" t="n">
         <v>1</v>
       </c>
-      <c r="O18" t="inlineStr"/>
       <c r="P18" t="inlineStr">
         <is>
           <t>CJDK3015677</t>
@@ -1931,7 +1914,6 @@
       <c r="N19" t="n">
         <v>1</v>
       </c>
-      <c r="O19" t="inlineStr"/>
       <c r="P19" t="inlineStr">
         <is>
           <t>CJQB3009764</t>
@@ -2011,7 +1993,6 @@
       <c r="N20" t="n">
         <v>1</v>
       </c>
-      <c r="O20" t="inlineStr"/>
       <c r="P20" t="inlineStr">
         <is>
           <t>CJKT3009929</t>
@@ -2091,7 +2072,6 @@
       <c r="N21" t="n">
         <v>1</v>
       </c>
-      <c r="O21" t="inlineStr"/>
       <c r="P21" t="inlineStr">
         <is>
           <t>CJWY2995765</t>
@@ -2171,7 +2151,6 @@
       <c r="N22" t="n">
         <v>1</v>
       </c>
-      <c r="O22" t="inlineStr"/>
       <c r="P22" t="inlineStr">
         <is>
           <t>CJJS2994644</t>
@@ -2251,7 +2230,6 @@
       <c r="N23" t="n">
         <v>1</v>
       </c>
-      <c r="O23" t="inlineStr"/>
       <c r="P23" t="inlineStr">
         <is>
           <t>CJQB2994598</t>
@@ -2331,7 +2309,6 @@
       <c r="N24" t="n">
         <v>1</v>
       </c>
-      <c r="O24" t="inlineStr"/>
       <c r="P24" t="inlineStr">
         <is>
           <t>CJTZ2983407</t>
@@ -2411,7 +2388,6 @@
       <c r="N25" t="n">
         <v>1</v>
       </c>
-      <c r="O25" t="inlineStr"/>
       <c r="P25" t="inlineStr">
         <is>
           <t>CJLY2977859</t>
@@ -2491,7 +2467,6 @@
       <c r="N26" t="n">
         <v>1</v>
       </c>
-      <c r="O26" t="inlineStr"/>
       <c r="P26" t="inlineStr">
         <is>
           <t>CJTZ2977891</t>
@@ -2571,7 +2546,6 @@
       <c r="N27" t="n">
         <v>1</v>
       </c>
-      <c r="O27" t="inlineStr"/>
       <c r="P27" t="inlineStr">
         <is>
           <t>CJTZ2975608</t>
@@ -2651,7 +2625,6 @@
       <c r="N28" t="n">
         <v>1</v>
       </c>
-      <c r="O28" t="inlineStr"/>
       <c r="P28" t="inlineStr">
         <is>
           <t>CJTZ2974582</t>
@@ -2731,7 +2704,6 @@
       <c r="N29" t="n">
         <v>1</v>
       </c>
-      <c r="O29" t="inlineStr"/>
       <c r="P29" t="inlineStr">
         <is>
           <t>CJTZ2974745</t>
@@ -2811,7 +2783,6 @@
       <c r="N30" t="n">
         <v>1</v>
       </c>
-      <c r="O30" t="inlineStr"/>
       <c r="P30" t="inlineStr">
         <is>
           <t>CJTZ2972533</t>
@@ -2891,7 +2862,6 @@
       <c r="N31" t="n">
         <v>1</v>
       </c>
-      <c r="O31" t="inlineStr"/>
       <c r="P31" t="inlineStr">
         <is>
           <t>CJMY2970588</t>
@@ -2971,7 +2941,6 @@
       <c r="N32" t="n">
         <v>1</v>
       </c>
-      <c r="O32" t="inlineStr"/>
       <c r="P32" t="inlineStr">
         <is>
           <t>CJLT2962050</t>
@@ -3051,7 +3020,6 @@
       <c r="N33" t="n">
         <v>1</v>
       </c>
-      <c r="O33" t="inlineStr"/>
       <c r="P33" t="inlineStr">
         <is>
           <t>CJWL2962205</t>
@@ -3131,7 +3099,6 @@
       <c r="N34" t="n">
         <v>1</v>
       </c>
-      <c r="O34" t="inlineStr"/>
       <c r="P34" t="inlineStr">
         <is>
           <t>CJLY2960883</t>
@@ -3211,7 +3178,6 @@
       <c r="N35" t="n">
         <v>1</v>
       </c>
-      <c r="O35" t="inlineStr"/>
       <c r="P35" t="inlineStr">
         <is>
           <t>CJTZ2959166</t>
@@ -3291,7 +3257,6 @@
       <c r="N36" t="n">
         <v>1</v>
       </c>
-      <c r="O36" t="inlineStr"/>
       <c r="P36" t="inlineStr">
         <is>
           <t>CJLY2959189</t>
@@ -3371,7 +3336,6 @@
       <c r="N37" t="n">
         <v>1</v>
       </c>
-      <c r="O37" t="inlineStr"/>
       <c r="P37" t="inlineStr">
         <is>
           <t>CJWL2959133</t>
@@ -3451,7 +3415,6 @@
       <c r="N38" t="n">
         <v>1</v>
       </c>
-      <c r="O38" t="inlineStr"/>
       <c r="P38" t="inlineStr">
         <is>
           <t>CJWL2959120</t>
@@ -3531,7 +3494,6 @@
       <c r="N39" t="n">
         <v>1</v>
       </c>
-      <c r="O39" t="inlineStr"/>
       <c r="P39" t="inlineStr">
         <is>
           <t>CJLY2956614</t>
@@ -3611,7 +3573,6 @@
       <c r="N40" t="n">
         <v>1</v>
       </c>
-      <c r="O40" t="inlineStr"/>
       <c r="P40" t="inlineStr">
         <is>
           <t>CJLT2956851</t>
@@ -3691,7 +3652,6 @@
       <c r="N41" t="n">
         <v>1</v>
       </c>
-      <c r="O41" t="inlineStr"/>
       <c r="P41" t="inlineStr">
         <is>
           <t>CJTZ2954056</t>
@@ -3771,7 +3731,6 @@
       <c r="N42" t="n">
         <v>1</v>
       </c>
-      <c r="O42" t="inlineStr"/>
       <c r="P42" t="inlineStr">
         <is>
           <t>CJWL2954034</t>
@@ -3851,7 +3810,6 @@
       <c r="N43" t="n">
         <v>1</v>
       </c>
-      <c r="O43" t="inlineStr"/>
       <c r="P43" t="inlineStr">
         <is>
           <t>CJLY2952354</t>
@@ -3931,7 +3889,6 @@
       <c r="N44" t="n">
         <v>1</v>
       </c>
-      <c r="O44" t="inlineStr"/>
       <c r="P44" t="inlineStr">
         <is>
           <t>CJWL2950701</t>
@@ -4011,7 +3968,6 @@
       <c r="N45" t="n">
         <v>1</v>
       </c>
-      <c r="O45" t="inlineStr"/>
       <c r="P45" t="inlineStr">
         <is>
           <t>CJQZ2950661</t>
@@ -4091,7 +4047,6 @@
       <c r="N46" t="n">
         <v>1</v>
       </c>
-      <c r="O46" t="inlineStr"/>
       <c r="P46" t="inlineStr">
         <is>
           <t>CJWL2950479</t>
@@ -4171,7 +4126,6 @@
       <c r="N47" t="n">
         <v>1</v>
       </c>
-      <c r="O47" t="inlineStr"/>
       <c r="P47" t="inlineStr">
         <is>
           <t>CJWL2949270</t>
@@ -4251,7 +4205,6 @@
       <c r="N48" t="n">
         <v>1</v>
       </c>
-      <c r="O48" t="inlineStr"/>
       <c r="P48" t="inlineStr">
         <is>
           <t>CJTZ2949455</t>
@@ -4331,7 +4284,6 @@
       <c r="N49" t="n">
         <v>1</v>
       </c>
-      <c r="O49" t="inlineStr"/>
       <c r="P49" t="inlineStr">
         <is>
           <t>CJTZ2949439</t>
@@ -4411,7 +4363,6 @@
       <c r="N50" t="n">
         <v>1</v>
       </c>
-      <c r="O50" t="inlineStr"/>
       <c r="P50" t="inlineStr">
         <is>
           <t>CJLY2949812</t>
@@ -4491,7 +4442,6 @@
       <c r="N51" t="n">
         <v>1</v>
       </c>
-      <c r="O51" t="inlineStr"/>
       <c r="P51" t="inlineStr">
         <is>
           <t>CJKT2949638</t>
@@ -4571,7 +4521,6 @@
       <c r="N52" t="n">
         <v>1</v>
       </c>
-      <c r="O52" t="inlineStr"/>
       <c r="P52" t="inlineStr">
         <is>
           <t>CJLY2950046</t>
@@ -4651,7 +4600,6 @@
       <c r="N53" t="n">
         <v>1</v>
       </c>
-      <c r="O53" t="inlineStr"/>
       <c r="P53" t="inlineStr">
         <is>
           <t>CJQZ2950122</t>
@@ -4731,7 +4679,6 @@
       <c r="N54" t="n">
         <v>1</v>
       </c>
-      <c r="O54" t="inlineStr"/>
       <c r="P54" t="inlineStr">
         <is>
           <t>CJLY2949916</t>
@@ -4811,7 +4758,6 @@
       <c r="N55" t="n">
         <v>1</v>
       </c>
-      <c r="O55" t="inlineStr"/>
       <c r="P55" t="inlineStr">
         <is>
           <t>CJKT2950130</t>
@@ -4891,7 +4837,6 @@
       <c r="N56" t="n">
         <v>1</v>
       </c>
-      <c r="O56" t="inlineStr"/>
       <c r="P56" t="inlineStr">
         <is>
           <t>CJLY2948751</t>
@@ -4971,7 +4916,6 @@
       <c r="N57" t="n">
         <v>1</v>
       </c>
-      <c r="O57" t="inlineStr"/>
       <c r="P57" t="inlineStr">
         <is>
           <t>CJKT2939320</t>
@@ -5051,7 +4995,6 @@
       <c r="N58" t="n">
         <v>1</v>
       </c>
-      <c r="O58" t="inlineStr"/>
       <c r="P58" t="inlineStr">
         <is>
           <t>CJWL2939272</t>
@@ -5131,7 +5074,6 @@
       <c r="N59" t="n">
         <v>1</v>
       </c>
-      <c r="O59" t="inlineStr"/>
       <c r="P59" t="inlineStr">
         <is>
           <t>CJJK2935423</t>
@@ -5211,7 +5153,6 @@
       <c r="N60" t="n">
         <v>1</v>
       </c>
-      <c r="O60" t="inlineStr"/>
       <c r="P60" t="inlineStr">
         <is>
           <t>CJTZ2935345</t>
@@ -5291,7 +5232,6 @@
       <c r="N61" t="n">
         <v>1</v>
       </c>
-      <c r="O61" t="inlineStr"/>
       <c r="P61" t="inlineStr">
         <is>
           <t>CJLY2934373</t>
@@ -5371,7 +5311,6 @@
       <c r="N62" t="n">
         <v>1</v>
       </c>
-      <c r="O62" t="inlineStr"/>
       <c r="P62" t="inlineStr">
         <is>
           <t>CJWL2934898</t>
@@ -5451,7 +5390,6 @@
       <c r="N63" t="n">
         <v>1</v>
       </c>
-      <c r="O63" t="inlineStr"/>
       <c r="P63" t="inlineStr">
         <is>
           <t>CJLT2934052</t>
@@ -5531,7 +5469,6 @@
       <c r="N64" t="n">
         <v>1</v>
       </c>
-      <c r="O64" t="inlineStr"/>
       <c r="P64" t="inlineStr">
         <is>
           <t>CJWL2935395</t>
@@ -5611,7 +5548,6 @@
       <c r="N65" t="n">
         <v>1</v>
       </c>
-      <c r="O65" t="inlineStr"/>
       <c r="P65" t="inlineStr">
         <is>
           <t>CJLY2935356</t>
@@ -5691,7 +5627,6 @@
       <c r="N66" t="n">
         <v>1</v>
       </c>
-      <c r="O66" t="inlineStr"/>
       <c r="P66" t="inlineStr">
         <is>
           <t>CJTZ2935432</t>
@@ -5771,7 +5706,6 @@
       <c r="N67" t="n">
         <v>1</v>
       </c>
-      <c r="O67" t="inlineStr"/>
       <c r="P67" t="inlineStr">
         <is>
           <t>CJTZ2935441</t>
@@ -5851,7 +5785,6 @@
       <c r="N68" t="n">
         <v>1</v>
       </c>
-      <c r="O68" t="inlineStr"/>
       <c r="P68" t="inlineStr">
         <is>
           <t>CJQZ2935408</t>
@@ -5931,7 +5864,6 @@
       <c r="N69" t="n">
         <v>1</v>
       </c>
-      <c r="O69" t="inlineStr"/>
       <c r="P69" t="inlineStr">
         <is>
           <t>CJKT2934384</t>
@@ -6011,7 +5943,6 @@
       <c r="N70" t="n">
         <v>1</v>
       </c>
-      <c r="O70" t="inlineStr"/>
       <c r="P70" t="inlineStr">
         <is>
           <t>CJWS2930927</t>
@@ -6091,7 +6022,6 @@
       <c r="N71" t="n">
         <v>1</v>
       </c>
-      <c r="O71" t="inlineStr"/>
       <c r="P71" t="inlineStr">
         <is>
           <t>CJKT2928545</t>
@@ -6105,6 +6035,1686 @@
       <c r="R71" t="inlineStr">
         <is>
           <t>2064585550960050178</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>z29d7djizwmm5v7321bqb71y</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>676716d67602c42f64f06f94</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Grey Grid Collision Black Sleeveless Waist Cinched A-line Short Suit Dress</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>https://cf.cjdropshipping.com/763ec58e-2fc0-4216-93c6-cf5e94ff3430.png,https://cf.cjdropshipping.com/46e7183b-5954-4096-868a-83c7736595ce.png</t>
+        </is>
+      </c>
+      <c r="E72" t="n">
+        <v>60</v>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>Step into sophistication with the Grey Grid Collision Black Sleeveless Waist Cinched A-line Short Suit Dress. Designed to flatter all body types, this modern piece combines a chic silhouette with stylish detailing. Perfect for any occasion, it effortlessly enhances your confidence and makes a bold statement wherever you go.</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>womens</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>Women's Clothing , Tops , Sets , Lady Dresses</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="J72" t="n">
+        <v>0</v>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>[['Gray-S', 'CJLY292811301AZ'], ['Gray-M', 'CJLY292811302BY'], ['Gray-L', 'CJLY292811303CX'], ['Gray-Xl', 'CJLY292811304DW'], ['Gray-2xl', 'CJLY292811305EV']]</t>
+        </is>
+      </c>
+      <c r="L72" t="n">
+        <v>243</v>
+      </c>
+      <c r="M72" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="N72" t="n">
+        <v>1</v>
+      </c>
+      <c r="O72" t="inlineStr"/>
+      <c r="P72" t="inlineStr">
+        <is>
+          <t>CJLY2928113</t>
+        </is>
+      </c>
+      <c r="Q72" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="R72" t="inlineStr">
+        <is>
+          <t>2064529979171561473</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>7a3h4yva09xokui0xb9whohz</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>676716d67602c42f64f06f94</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Gray Half-zip Waist-cinching Pleated Hoodie Dress</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>https://cf.cjdropshipping.com/0cfcab34-92fe-46af-945f-467cc909fec6.jpg,https://cf.cjdropshipping.com/19cb9f52-4b04-44d0-b670-b6afdd9846b3.jpg,https://oss-cf.cjdropshipping.com/product/2026/07/17/08/5cfce949-887d-4176-9a1e-12e2539fe938.jpg,https://oss-cf.cjdropshipping.com/product/2026/07/17/08/84fb5b07-b394-4cea-8bea-b2bb6895146d.jpg</t>
+        </is>
+      </c>
+      <c r="E73" t="n">
+        <v>72</v>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>Experience comfort and style with our Gray Half-zip Waist-cinching Pleated Hoodie Dress. This versatile piece features a flattering silhouette, adjustable waist for a customized fit, and pleated detailing for added flair. Perfect for casual outings or lounging at home, it combines practicality with fashion effortlessly. Upgrade your wardrobe today!</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>womens</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>Women's Clothing , Tops , Sets , Lady Dresses</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="J73" t="n">
+        <v>0</v>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>[['Gray-S', 'CJLY292824201AZ'], ['Gray-M', 'CJLY292824202BY'], ['Gray-L', 'CJLY292824203CX'], ['Gray-XL', 'CJLY292824204DW'], ['Gray-XXL', 'CJLY292824205EV'], ['Light Khaki-S', 'CJLY292824206FU'], ['Light Khaki-M', 'CJLY292824207GT'], ['Light Khaki-L', 'CJLY292824208HS'], ['Light Khaki-XL', 'CJLY292824209IR'], ['Light Khaki-XXL', 'CJLY292824210JQ'], ['Pink-S', 'CJLY292824211KP'], ['Pink-M', 'CJLY292824212LO'], ['Pink-L', 'CJLY292824213MN'], ['Pink-XL', 'CJLY292824214NM'], ['Pink-XXL', 'CJLY292824215OL']]</t>
+        </is>
+      </c>
+      <c r="L73" t="n">
+        <v>477</v>
+      </c>
+      <c r="M73" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="N73" t="n">
+        <v>1</v>
+      </c>
+      <c r="O73" t="inlineStr"/>
+      <c r="P73" t="inlineStr">
+        <is>
+          <t>CJLY2928242</t>
+        </is>
+      </c>
+      <c r="Q73" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="R73" t="inlineStr">
+        <is>
+          <t>2064541723226324993</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>03llnq6gopdlp4eytgviscuu</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>676716d67602c42f64f06f94</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Women's Solid Color Lapel Zip Pullover Sweater, Loose 3D Casual Top For Autumn</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>https://cf.cjdropshipping.com/3836e342-893b-4d9d-b32c-b50f806c438b.jpg,https://cf.cjdropshipping.com/8c09029a-3d57-496f-8b7f-7a6d0a13b6e3.jpg,https://cf.cjdropshipping.com/a138394b-681f-4bff-90a9-df49b002280b.jpg,https://cf.cjdropshipping.com/e4ea24dc-554c-4558-b420-100a6f42289a.jpg,https://cf.cjdropshipping.com/2abd05cf-a8f7-4b4e-9b44-18ce9e952a46.jpg,https://cf.cjdropshipping.com/0c10f83a-bce8-438b-bbe7-43aba62c047e.jpg,https://cf.cjdropshipping.com/72e66f42-96ac-42b2-9cd7-5ee9e6b7bc9a.jpg,https://cf.cjdropshipping.com/86d4d04f-0cf5-4656-b1f5-f638da9d06dd.jpg,https://cf.cjdropshipping.com/67096893-bfa5-4171-aac1-c18aee2a9684.jpg,https://cf.cjdropshipping.com/d3fbcb2b-975a-4760-8bea-48df25e2d9d6.jpg</t>
+        </is>
+      </c>
+      <c r="E74" t="n">
+        <v>77.90000000000001</v>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>Stay cozy and stylish this autumn with our Women’s Solid Color Lapel Zip Pullover Sweater. This loose-fitting, 3D casual top offers unmatched comfort and versatility. Perfect for layering or wearing solo, it effortlessly complements your wardrobe, making it an essential piece for chilly days. Embrace warmth while looking fabulous!</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>womens</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>Women's Clothing , Tops , Sets , Sweaters</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="J74" t="n">
+        <v>2</v>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>[['Sky Blue-S', 'CJMY292781301AZ'], ['Sky Blue-M', 'CJMY292781302BY'], ['Sky Blue-L', 'CJMY292781303CX'], ['Sky Blue-XL', 'CJMY292781304DW'], ['Sky Blue-XXL', 'CJMY292781305EV'], ['Sky Blue-XXXL', 'CJMY292781306FU'], ['OffWhite-S', 'CJMY292781307GT'], ['OffWhite-M', 'CJMY292781308HS'], ['OffWhite-L', 'CJMY292781309IR'], ['OffWhite-XL', 'CJMY292781310JQ'], ['OffWhite-XXL', 'CJMY292781311KP'], ['OffWhite-XXXL', 'CJMY292781312LO'], ['Army Green-S', 'CJMY292781313MN'], ['Army Green-M', 'CJMY292781314NM'], ['Army Green-L', 'CJMY292781315OL'], ['Army Green-XL', 'CJMY292781316PK'], ['Army Green-XXL', 'CJMY292781317QJ'], ['Army Green-XXXL', 'CJMY292781318RI'], ['Light Green-S', 'CJMY292781319SH'], ['Light Green-M', 'CJMY292781320TG'], ['Light Green-L', 'CJMY292781321UF'], ['Light Green-XL', 'CJMY292781322VE'], ['Light Green-XXL', 'CJMY292781323WD'], ['Light Green-XXXL', 'CJMY292781324XC'], ['Black-S', 'CJMY292781325YB'], ['Black-M', 'CJMY292781326ZA'], ['Black-L', 'CJMY292781327AZ'], ['Black-XL', 'CJMY292781328BY'], ['Black-XXL', 'CJMY292781329CX'], ['Black-XXXL', 'CJMY292781330DW'], ['Coffee-S', 'CJMY292781331EV'], ['Coffee-M', 'CJMY292781332FU'], ['Coffee-L', 'CJMY292781333GT'], ['Coffee-XL', 'CJMY292781334HS'], ['Coffee-XXL', 'CJMY292781335IR'], ['Coffee-XXXL', 'CJMY292781336JQ'], ['Grey-S', 'CJMY292781337KP'], ['Grey-M', 'CJMY292781338LO'], ['Grey-L', 'CJMY292781339MN'], ['Grey-XL', 'CJMY292781340NM'], ['Grey-XXL', 'CJMY292781341OL'], ['Grey-XXXL', 'CJMY292781342PK'], ['Pink-S', 'CJMY292781343QJ'], ['Pink-M', 'CJMY292781344RI'], ['Pink-L', 'CJMY292781345SH'], ['Pink-XL', 'CJMY292781346TG'], ['Pink-XXL', 'CJMY292781347UF'], ['Pink-XXXL', 'CJMY292781348VE'], ['Purple-S', 'CJMY292781349WD'], ['Purple-M', 'CJMY292781350XC'], ['Purple-L', 'CJMY292781351YB'], ['Purple-XL', 'CJMY292781352ZA'], ['Purple-XXL', 'CJMY292781353AZ'], ['Purple-XXXL', 'CJMY292781354BY'], ['Camel-S', 'CJMY292781355CX'], ['Camel-M', 'CJMY292781356DW'], ['Camel-L', 'CJMY292781357EV'], ['Camel-XL', 'CJMY292781358FU'], ['Camel-XXL', 'CJMY292781359GT'], ['Camel-XXXL', 'CJMY292781360HS']]</t>
+        </is>
+      </c>
+      <c r="L74" t="n">
+        <v>500</v>
+      </c>
+      <c r="M74" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="N74" t="n">
+        <v>1</v>
+      </c>
+      <c r="O74" t="inlineStr"/>
+      <c r="P74" t="inlineStr">
+        <is>
+          <t>CJMY2927813</t>
+        </is>
+      </c>
+      <c r="Q74" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="R74" t="inlineStr">
+        <is>
+          <t>2064344886167896065</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>j27dy61t82ntkyqyzzzbbby9</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>676716d67602c42f64f06f94</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Color Block Star Print Rib Collar Snap Button Longline Varsity Baseball Jacket</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>https://cf.cjdropshipping.com/9650fffc-1527-4c81-997d-2933985d45a6.jpg,https://cf.cjdropshipping.com/ffb29f9a-1168-4dcc-880a-19187b18e9a5.jpg,https://cf.cjdropshipping.com/b8d2638b-39bf-4809-9b82-274e005346e2.jpg</t>
+        </is>
+      </c>
+      <c r="E75" t="n">
+        <v>78.8</v>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>Step up your style with our Color Block Star Print Rib Collar Snap Button Longline Varsity Baseball Jacket. This trendy outerwear combines bold colors and a striking star print, perfect for making a statement. Its comfortable fit and sporty design effortlessly enhance any casual outfit, making it a must-have for fashion lovers.</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>womens</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>Women's Clothing , Tops , Sets , Suits , Sets</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="J75" t="n">
+        <v>0</v>
+      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>[['Green-S', 'CJTZ292747801AZ'], ['Green-M', 'CJTZ292747802BY'], ['Green-L', 'CJTZ292747803CX'], ['Green-Xl', 'CJTZ292747804DW'], ['Green-Xxl', 'CJTZ292747805EV']]</t>
+        </is>
+      </c>
+      <c r="L75" t="n">
+        <v>460</v>
+      </c>
+      <c r="M75" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="N75" t="n">
+        <v>1</v>
+      </c>
+      <c r="O75" t="inlineStr"/>
+      <c r="P75" t="inlineStr">
+        <is>
+          <t>CJTZ2927478</t>
+        </is>
+      </c>
+      <c r="Q75" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="R75" t="inlineStr">
+        <is>
+          <t>2064239006151770114</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>5livktiv2na72bknd4lra4hb</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>676716d67602c42f64f06f94</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Military Green Side Drawstring Loose Seven Quarter Sleeve T-shirt Short Skirt</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>https://cf.cjdropshipping.com/4c3f6b8a-d4fc-4a65-8cd0-f49e0e1e7e0d.png,https://cf.cjdropshipping.com/2aade528-c014-4c9a-b270-46c7a35efcd4.png</t>
+        </is>
+      </c>
+      <c r="E76" t="n">
+        <v>55.9</v>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>Discover ultimate comfort and style with our Military Green Side Drawstring Loose Seven Quarter Sleeve T-shirt Short Skirt. This versatile outfit combines casual elegance and practicality, perfect for any occasion. The adjustable drawstring allows for a customizable fit, while the trendy design ensures you remain fashionable and relaxed all day long.</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>womens</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>Women's Clothing , Tops , Sets , Lady Dresses</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="J76" t="n">
+        <v>0</v>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>[['Green-S', 'CJLY292713301AZ'], ['Green-M', 'CJLY292713302BY'], ['Green-L', 'CJLY292713303CX'], ['Green-Xl', 'CJLY292713304DW'], ['Green-2xl', 'CJLY292713305EV']]</t>
+        </is>
+      </c>
+      <c r="L76" t="n">
+        <v>300</v>
+      </c>
+      <c r="M76" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="N76" t="n">
+        <v>1</v>
+      </c>
+      <c r="O76" t="inlineStr"/>
+      <c r="P76" t="inlineStr">
+        <is>
+          <t>CJLY2927133</t>
+        </is>
+      </c>
+      <c r="Q76" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="R76" t="inlineStr">
+        <is>
+          <t>2064205372002062338</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>3m4x45jlxw0bsfam0p4qq9qc</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>676716d67602c42f64f06f94</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>One Shoulder Bubble Sleeve Black Lace Patchwork Red Short Dress</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>https://cf.cjdropshipping.com/7669e640-8c49-4288-9e02-2ea86ae5a7ee.png,https://cf.cjdropshipping.com/63d3f1b4-4cd7-4a68-bb0e-0a7f85376263.png,https://cf.cjdropshipping.com/67d5449c-57e8-46d9-8b17-6fa6945c6c75.png</t>
+        </is>
+      </c>
+      <c r="E77" t="n">
+        <v>65</v>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>Step into elegance with our One Shoulder Bubble Sleeve Black Lace Patchwork Red Short Dress. Featuring a chic asymmetrical design and luxurious lace detailing, this dress is perfect for making a statement at any event. Its vibrant hue and playful silhouette ensure all eyes will be on you. Embrace your bold side!</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>womens</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>Women's Clothing , Tops , Sets , Lady Dresses</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="J77" t="n">
+        <v>0</v>
+      </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>[['Red-S', 'CJLY292333101AZ'], ['Red-M', 'CJLY292333102BY'], ['Red-L', 'CJLY292333103CX'], ['Red-Xl', 'CJLY292333104DW'], ['Red-2xl', 'CJLY292333105EV']]</t>
+        </is>
+      </c>
+      <c r="L77" t="n">
+        <v>180</v>
+      </c>
+      <c r="M77" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="N77" t="n">
+        <v>1</v>
+      </c>
+      <c r="O77" t="inlineStr"/>
+      <c r="P77" t="inlineStr">
+        <is>
+          <t>CJLY2923331</t>
+        </is>
+      </c>
+      <c r="Q77" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="R77" t="inlineStr">
+        <is>
+          <t>2062838654164832257</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>xzrydi9v0x7amezkw0pq6kkz</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>676716d67602c42f64f06f94</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>V-neck Sleeveless Linen Top &amp; Drawstring Shorts Set</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>https://cf.cjdropshipping.com/ba795410-1b1e-43ae-b0a9-fc04348c57df.png,https://cf.cjdropshipping.com/ed0b6104-fc19-4a68-8484-eda03f059360.png</t>
+        </is>
+      </c>
+      <c r="E78" t="n">
+        <v>56.5</v>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>Embrace effortless style with our V-neck Sleeveless Linen Top &amp; Drawstring Shorts Set. Perfect for warm days, this breathable ensemble blends comfort and chic sophistication. The relaxed fit flatters every silhouette, while the versatile design allows for endless styling options. Stay cool and fashionable all summer long with this must-have outfit!</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>womens</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>Women's Clothing , Tops , Sets , Suits , Sets</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="J78" t="n">
+        <v>1</v>
+      </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>[['Offwhite-S', 'CJTZ292238801AZ'], ['Offwhite-M', 'CJTZ292238802BY'], ['Offwhite-L', 'CJTZ292238803CX'], ['Offwhite-XL', 'CJTZ292238804DW'], ['Offwhite-2XL', 'CJTZ292238805EV']]</t>
+        </is>
+      </c>
+      <c r="L78" t="n">
+        <v>251</v>
+      </c>
+      <c r="M78" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="N78" t="n">
+        <v>1</v>
+      </c>
+      <c r="O78" t="inlineStr"/>
+      <c r="P78" t="inlineStr">
+        <is>
+          <t>CJTZ2922388</t>
+        </is>
+      </c>
+      <c r="Q78" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="R78" t="inlineStr">
+        <is>
+          <t>2062715584822607874</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>ogky1xyn8espqa6i65vlmo39</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>676716d67602c42f64f06f94</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Polo Collar Yellow White Plaid Short Sleeve Romper</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>https://cf.cjdropshipping.com/c18f716c-3bdf-4286-8511-d28a165d040d.png,https://cf.cjdropshipping.com/1159a077-f685-44af-b4b8-626b283439bb.png</t>
+        </is>
+      </c>
+      <c r="E79" t="n">
+        <v>46.3</v>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>Introducing our Polo Collar Yellow White Plaid Short Sleeve Romper! This stylish romper combines comfort and flair, perfect for sunny outings. Its vibrant plaid pattern adds a playful touch, while the short sleeves keep you cool. Effortlessly chic, it’s an ideal choice for casual gatherings or lounging in style!</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>womens</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>Women's Clothing , Tops , Sets , Rompers</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="J79" t="n">
+        <v>0</v>
+      </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>[['Yellow-S', 'CJLT292067001AZ'], ['Yellow-M', 'CJLT292067002BY'], ['Yellow-L', 'CJLT292067003CX'], ['Yellow-XL', 'CJLT292067004DW'], ['Yellow-2XL', 'CJLT292067005EV']]</t>
+        </is>
+      </c>
+      <c r="L79" t="n">
+        <v>312</v>
+      </c>
+      <c r="M79" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="N79" t="n">
+        <v>1</v>
+      </c>
+      <c r="O79" t="inlineStr"/>
+      <c r="P79" t="inlineStr">
+        <is>
+          <t>CJLT2920670</t>
+        </is>
+      </c>
+      <c r="Q79" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="R79" t="inlineStr">
+        <is>
+          <t>2062349378625118209</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>95t5znorpxw3ix1b6qhym87n</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>676716d67602c42f64f06f94</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Black Small High Neck Short Sleeved Slim Fit Professional Dress With Hip Hugging Design</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>https://cf.cjdropshipping.com/c66d380c-9187-4bcf-973d-7a77f3f69e25.png,https://cf.cjdropshipping.com/12e8129a-1828-4503-a6b9-30c40931ad88.png</t>
+        </is>
+      </c>
+      <c r="E80" t="n">
+        <v>68.5</v>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>Step into sophistication with our Black Small High Neck Short Sleeved Slim Fit Professional Dress. Featuring a stunning hip-hugging design, this dress effortlessly combines elegance with comfort. Perfect for the office or after hours, it accentuates your curves and makes a stylish statement. Elevate your wardrobe and shine on any occasion!</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>womens</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>Women's Clothing , Tops , Sets , Lady Dresses</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="J80" t="n">
+        <v>1</v>
+      </c>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>[['Black-S', 'CJLY292186401AZ'], ['Black-M', 'CJLY292186402BY'], ['Black-L', 'CJLY292186403CX'], ['Black-Xl', 'CJLY292186404DW'], ['Black-2xl', 'CJLY292186405EV']]</t>
+        </is>
+      </c>
+      <c r="L80" t="n">
+        <v>186</v>
+      </c>
+      <c r="M80" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="N80" t="n">
+        <v>1</v>
+      </c>
+      <c r="O80" t="inlineStr"/>
+      <c r="P80" t="inlineStr">
+        <is>
+          <t>CJLY2921864</t>
+        </is>
+      </c>
+      <c r="Q80" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="R80" t="inlineStr">
+        <is>
+          <t>2062473459822686210</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>sgmbohhlfevpssmplm2szolv</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>676716d67602c42f64f06f94</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Mibai Collision Black Border Hanging Neck Linen Long Vacation Dress</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>https://cf.cjdropshipping.com/f8c22b17-a8c5-40af-98f4-06fdef5907e9.png,https://cf.cjdropshipping.com/aacd7ef0-72e8-4468-b1eb-57d79a1dba42.png</t>
+        </is>
+      </c>
+      <c r="E81" t="n">
+        <v>60</v>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>Discover the Mibai Collision Black Border Hanging Neck Linen Long Vacation Dress, perfect for your summer getaway. Crafted from breathable linen with a stylish design, it ensures comfort and elegance. The eye-catching black border adds sophistication, making it a must-have for effortless beach strolls or chic evening outings. Unleash your style!</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>womens</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>Women's Clothing , Tops , Sets , Lady Dresses</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="J81" t="n">
+        <v>0</v>
+      </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>[['Beige-S', 'CJLY292188501AZ'], ['Beige-M', 'CJLY292188502BY'], ['Beige-L', 'CJLY292188503CX'], ['Beige-Xl', 'CJLY292188504DW'], ['Beige-2xl', 'CJLY292188505EV']]</t>
+        </is>
+      </c>
+      <c r="L81" t="n">
+        <v>289</v>
+      </c>
+      <c r="M81" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="N81" t="n">
+        <v>1</v>
+      </c>
+      <c r="O81" t="inlineStr"/>
+      <c r="P81" t="inlineStr">
+        <is>
+          <t>CJLY2921885</t>
+        </is>
+      </c>
+      <c r="Q81" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="R81" t="inlineStr">
+        <is>
+          <t>2062475444236754946</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>8pxvnwpj2ks0tc3w0y3w51x2</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>676716d67602c42f64f06f94</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Hanging Neck Deep V-fold Split Vacation Long Dress</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>https://cf.cjdropshipping.com/2932268b-c145-42e2-bc91-307ab719dbb0.png,https://cf.cjdropshipping.com/c2a53f58-3d26-4215-b0d8-6ba6eeeb085b.png</t>
+        </is>
+      </c>
+      <c r="E82" t="n">
+        <v>70.2</v>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>Step into summer with our Hanging Neck Deep V-fold Split Vacation Long Dress. This stunning piece combines elegance and comfort, featuring a flattering deep V neckline and chic split design. Perfect for beach days or evening strolls, it effortlessly enhances your silhouette. Embrace style and confidence on your next getaway!</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>womens</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>Women's Clothing , Tops , Sets , Lady Dresses</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="J82" t="n">
+        <v>1</v>
+      </c>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>[['Haze Blue-S', 'CJLY292034901AZ'], ['Haze Blue-M', 'CJLY292034902BY'], ['Haze Blue-L', 'CJLY292034903CX'], ['Haze Blue-Xl', 'CJLY292034904DW'], ['Haze Blue-2xl', 'CJLY292034905EV']]</t>
+        </is>
+      </c>
+      <c r="L82" t="n">
+        <v>359</v>
+      </c>
+      <c r="M82" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="N82" t="n">
+        <v>1</v>
+      </c>
+      <c r="O82" t="inlineStr"/>
+      <c r="P82" t="inlineStr">
+        <is>
+          <t>CJLY2920349</t>
+        </is>
+      </c>
+      <c r="Q82" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="R82" t="inlineStr">
+        <is>
+          <t>2062109525210071041</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>y308odbntu4jvtppzafvkgxc</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>676716d67602c42f64f06f94</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Tibetan Blue And White Pleated Hem Long Sleeved Waist Cinching Short Dress</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>https://cf.cjdropshipping.com/96a2356f-9041-456c-a22a-6a4ce8672b9e.png,https://cf.cjdropshipping.com/fd0674b6-136d-4b8a-9da1-471330e4f56f.png</t>
+        </is>
+      </c>
+      <c r="E83" t="n">
+        <v>77</v>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>Unveil your elegance with the Tibetan Blue and White Pleated Hem Long Sleeved Dress. This stunning garment features a flattering waist-cinching design and delicate pleats, perfect for any occasion. Embrace your unique style and make a statement wherever you go. Comfortable and chic, this dress is a must-have addition to your wardrobe!</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>womens</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>Women's Clothing , Tops , Sets , Lady Dresses</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="J83" t="n">
+        <v>0</v>
+      </c>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t>[['Navy blue-S', 'CJLY292036801AZ'], ['Navy blue-M', 'CJLY292036802BY'], ['Navy blue-L', 'CJLY292036803CX'], ['Navy blue-Xl', 'CJLY292036804DW'], ['Navy blue-2xl', 'CJLY292036805EV']]</t>
+        </is>
+      </c>
+      <c r="L83" t="n">
+        <v>420</v>
+      </c>
+      <c r="M83" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="N83" t="n">
+        <v>1</v>
+      </c>
+      <c r="O83" t="inlineStr"/>
+      <c r="P83" t="inlineStr">
+        <is>
+          <t>CJLY2920368</t>
+        </is>
+      </c>
+      <c r="Q83" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="R83" t="inlineStr">
+        <is>
+          <t>2062112052915765250</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>pu2u1z1qspifztawzd53cbrf</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>676716d67602c42f64f06f94</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Cream &amp; Brown Trim Sleeveless Linen Top &amp; Shorts Set</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>https://cf.cjdropshipping.com/ba263f77-287b-4354-a98e-981f110aa38b.png,https://cf.cjdropshipping.com/353f6415-525c-4eeb-8a93-b7609bc6f575.png</t>
+        </is>
+      </c>
+      <c r="E84" t="n">
+        <v>72</v>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>Upgrade your summer wardrobe with our Cream &amp; Brown Trim Sleeveless Linen Top &amp; Shorts Set. This chic ensemble combines comfort and style, featuring breathable linen fabric and a flattering fit. Perfect for casual outings or beach days, it exudes effortless sophistication. Embrace warm weather with this must-have addition!</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>womens</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>Women's Clothing , Tops , Sets , Suits , Sets</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="J84" t="n">
+        <v>0</v>
+      </c>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t>[['Cream Off White-S', 'CJTZ291903401AZ'], ['Cream Off White-M', 'CJTZ291903402BY'], ['Cream Off White-L', 'CJTZ291903403CX'], ['Cream Off White-XL', 'CJTZ291903404DW'], ['Cream Off White-2XL', 'CJTZ291903405EV']]</t>
+        </is>
+      </c>
+      <c r="L84" t="n">
+        <v>255</v>
+      </c>
+      <c r="M84" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="N84" t="n">
+        <v>1</v>
+      </c>
+      <c r="O84" t="inlineStr"/>
+      <c r="P84" t="inlineStr">
+        <is>
+          <t>CJTZ2919034</t>
+        </is>
+      </c>
+      <c r="Q84" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="R84" t="inlineStr">
+        <is>
+          <t>2062006174329626626</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>fbzgusbk5zq34mktkybn34ps</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>676716d67602c42f64f06f94</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Contrast-color Neck-hanging Linen Set</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>https://cf.cjdropshipping.com/7794ea88-fb99-43ac-9d65-49f0b2362a64.jpg,https://cf.cjdropshipping.com/0f2748a0-c695-4ee7-91c6-839b2246cafa.jpg</t>
+        </is>
+      </c>
+      <c r="E85" t="n">
+        <v>56.5</v>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>Introducing the Contrast-color Neck-hanging Linen Set, a stylish blend of comfort and elegance. Crafted from high-quality linen, this unique design features vibrant contrast colors, perfect for adding flair to your wardrobe. Lightweight and breathable, it's ideal for any occasion. Upgrade your fashion game and make a statement today!</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>womens</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>Women's Clothing , Tops , Sets , Suits , Sets</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="J85" t="n">
+        <v>0</v>
+      </c>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>[['White-S', 'CJTZ291780801AZ'], ['White-M', 'CJTZ291780802BY'], ['White-L', 'CJTZ291780803CX'], ['White-XL', 'CJTZ291780804DW'], ['White-XXL', 'CJTZ291780805EV']]</t>
+        </is>
+      </c>
+      <c r="L85" t="n">
+        <v>250</v>
+      </c>
+      <c r="M85" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="N85" t="n">
+        <v>1</v>
+      </c>
+      <c r="O85" t="inlineStr"/>
+      <c r="P85" t="inlineStr">
+        <is>
+          <t>CJTZ2917808</t>
+        </is>
+      </c>
+      <c r="Q85" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="R85" t="inlineStr">
+        <is>
+          <t>2061640561325268993</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>jaqz0ylsxh4w58eh9lwnowfh</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>676716d67602c42f64f06f94</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Black &amp; White Striped Halter Knit Romper</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>https://cf.cjdropshipping.com/0ba5d596-7e6c-411c-8868-2f1948530e17.png,https://cf.cjdropshipping.com/61c6dce6-5b75-425d-aeda-ed02107c480f.png</t>
+        </is>
+      </c>
+      <c r="E86" t="n">
+        <v>30.8</v>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>Step into style with our Black &amp; White Striped Halter Knit Romper! This chic piece features a trendy halter neck and comfortable fabric, perfect for casual outings or beach days. Its striking design adds flair to any wardrobe, ensuring you stand out effortlessly. Embrace fashion with this must-have romper!</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>womens</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>Women's Clothing , Tops , Sets , Rompers</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="J86" t="n">
+        <v>1</v>
+      </c>
+      <c r="K86" t="inlineStr">
+        <is>
+          <t>[['Black  White-S', 'CJLT291788501AZ'], ['Black  White-M', 'CJLT291788502BY'], ['Black  White-L', 'CJLT291788503CX'], ['Black  White-XL', 'CJLT291788504DW'], ['Black  White-2XL', 'CJLT291788505EV']]</t>
+        </is>
+      </c>
+      <c r="L86" t="n">
+        <v>188</v>
+      </c>
+      <c r="M86" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="N86" t="n">
+        <v>1</v>
+      </c>
+      <c r="O86" t="inlineStr"/>
+      <c r="P86" t="inlineStr">
+        <is>
+          <t>CJLT2917885</t>
+        </is>
+      </c>
+      <c r="Q86" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="R86" t="inlineStr">
+        <is>
+          <t>2061648721459896321</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>7j4rwuy0bdq871ovg28plal6</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>676716d67602c42f64f06f94</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Black And White Vertical Stripe V-neck Sleeveless Patchwork Ruffle Edge Dress</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>https://cf.cjdropshipping.com/ad622daf-a6c7-414b-8d92-55996763fd0a.png,https://cf.cjdropshipping.com/e6923bde-5a47-4782-9655-a643c3875f15.png</t>
+        </is>
+      </c>
+      <c r="E87" t="n">
+        <v>68.5</v>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>Step into style with the Black and White Vertical Stripe V-neck Sleeveless Patchwork Ruffle Edge Dress. This chic design combines playful ruffles with a flattering V-neck, perfect for any occasion. Its bold stripes and unique patchwork details ensure you stand out effortlessly, making it a must-have addition to your wardrobe.</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>womens</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>Women's Clothing , Tops , Sets , Lady Dresses</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="J87" t="n">
+        <v>0</v>
+      </c>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t>[['White-S', 'CJLY291734601AZ'], ['White-M', 'CJLY291734602BY'], ['White-L', 'CJLY291734603CX'], ['White-Xl', 'CJLY291734604DW'], ['White-2xl', 'CJLY291734605EV']]</t>
+        </is>
+      </c>
+      <c r="L87" t="n">
+        <v>183</v>
+      </c>
+      <c r="M87" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="N87" t="n">
+        <v>1</v>
+      </c>
+      <c r="O87" t="inlineStr"/>
+      <c r="P87" t="inlineStr">
+        <is>
+          <t>CJLY2917346</t>
+        </is>
+      </c>
+      <c r="Q87" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="R87" t="inlineStr">
+        <is>
+          <t>2061371030694547458</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>m6prkynu8wxhv2p2ol58ozzb</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>676716d67602c42f64f06f94</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Green Short-sleeved Shirt And Wide-leg Pants Set</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>https://oss-cf.cjdropshipping.com/product/2026/06/15/02/f223fc63-da54-40b2-887b-760c61c7ad0e.jpg,https://oss-cf.cjdropshipping.com/product/2026/06/15/02/ae602353-b0e9-43f4-8452-c8eeaca1d72f.jpg</t>
+        </is>
+      </c>
+      <c r="E88" t="n">
+        <v>85.7</v>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>Stylish and comfortable, the Green Short-sleeved Shirt and Wide-leg Pants Set is perfect for every occasion. This chic ensemble features breathable fabric and a relaxed fit, ensuring you stay fashionable while feeling at ease. Pair it with your favorite accessories for a stunning summer look that turns heads wherever you go!</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>womens</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>Women's Clothing , Tops , Sets , Suits , Sets</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="J88" t="n">
+        <v>2</v>
+      </c>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>[['Green-S', 'CJTZ291672301AZ'], ['Green-M', 'CJTZ291672302BY'], ['Green-L', 'CJTZ291672303CX'], ['Green-XL', 'CJTZ291672304DW'], ['Green-XXL', 'CJTZ291672305EV']]</t>
+        </is>
+      </c>
+      <c r="L88" t="n">
+        <v>393</v>
+      </c>
+      <c r="M88" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="N88" t="n">
+        <v>1</v>
+      </c>
+      <c r="O88" t="inlineStr"/>
+      <c r="P88" t="inlineStr">
+        <is>
+          <t>CJTZ2916723</t>
+        </is>
+      </c>
+      <c r="Q88" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="R88" t="inlineStr">
+        <is>
+          <t>2061258621743681538</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>zfhvpr5sqztjccwf6cxz7jc7</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>676716d67602c42f64f06f94</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Lake Blue Cross Hanging Neck And Waist A-line Medium Length Dress</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>https://cf.cjdropshipping.com/bb289e38-6682-4ba6-b4eb-470cb889f00a.png,https://cf.cjdropshipping.com/4e1cc535-7728-4774-8191-a61da59e9a5c.png</t>
+        </is>
+      </c>
+      <c r="E89" t="n">
+        <v>77</v>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>Immerse yourself in effortless elegance with our Lake Blue Cross Hanging Neck and Waist A-Line Dress. This medium-length masterpiece combines style and comfort, featuring a stunning cross neckline and flattering A-line silhouette. Perfect for any occasion, this dress will make you feel confident and radiant. Embrace sophistication today!</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>womens</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>Women's Clothing , Tops , Sets , Lady Dresses</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="J89" t="n">
+        <v>0</v>
+      </c>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>[['Blue-S', 'CJLY291746101AZ'], ['Blue-M', 'CJLY291746102BY'], ['Blue-L', 'CJLY291746103CX'], ['Blue-Xl', 'CJLY291746104DW'], ['Blue-2xl', 'CJLY291746105EV']]</t>
+        </is>
+      </c>
+      <c r="L89" t="n">
+        <v>488</v>
+      </c>
+      <c r="M89" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="N89" t="n">
+        <v>1</v>
+      </c>
+      <c r="O89" t="inlineStr"/>
+      <c r="P89" t="inlineStr">
+        <is>
+          <t>CJLY2917461</t>
+        </is>
+      </c>
+      <c r="Q89" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="R89" t="inlineStr">
+        <is>
+          <t>2061385035872821250</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>kb4m2t69f4gtdcglit611n93</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>676716d67602c42f64f06f94</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Half-zip Stand-up Collar Hoodie Dress</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>https://cf.cjdropshipping.com/315f05a4-646c-43b7-846c-d5ee0864c549.jpg,https://cf.cjdropshipping.com/b24e3622-8088-439c-b8e3-b5787300b55d.jpg</t>
+        </is>
+      </c>
+      <c r="E90" t="n">
+        <v>61.7</v>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>Upgrade your casual wardrobe with our Half-zip Stand-up Collar Hoodie Dress. This chic and versatile piece combines comfort and style, perfect for any occasion. Featuring a cozy hood and adjustable zipper, it offers an effortless look. Pair it with sneakers or boots for a trendy outfit you’ll love wearing!</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>womens</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>Women's Clothing , Tops , Sets , Lady Dresses</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="J90" t="n">
+        <v>1</v>
+      </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>[['Brown-S', 'CJLY291687901AZ'], ['Brown-M', 'CJLY291687902BY'], ['Brown-L', 'CJLY291687903CX'], ['Brown-XL', 'CJLY291687904DW'], ['Brown-XXL', 'CJLY291687905EV']]</t>
+        </is>
+      </c>
+      <c r="L90" t="n">
+        <v>450</v>
+      </c>
+      <c r="M90" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="N90" t="n">
+        <v>1</v>
+      </c>
+      <c r="O90" t="inlineStr"/>
+      <c r="P90" t="inlineStr">
+        <is>
+          <t>CJLY2916879</t>
+        </is>
+      </c>
+      <c r="Q90" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="R90" t="inlineStr">
+        <is>
+          <t>2061286644921114626</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>3wdwrs1sd7sujac38cb1a21j</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>676716d67602c42f64f06f94</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Black Satin Lace-Trim V-Neck Top &amp; Skirt Set</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>https://cf.cjdropshipping.com/c5121122-947d-4a7d-ac7b-704c8cdb7e89.jpg,https://cf.cjdropshipping.com/85c00822-ad44-4446-b9a5-b8138ef5a644.png</t>
+        </is>
+      </c>
+      <c r="E91" t="n">
+        <v>54.8</v>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>Introducing the Black Satin Lace-Trim V-Neck Top &amp; Skirt Set, a stunning ensemble designed for sophistication. The luxurious satin fabric flows gracefully, complemented by delicate lace trim for an exquisite touch. Perfect for any occasion, this set effortlessly combines elegance and comfort, ensuring you turn heads wherever you go.</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>womens</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>Women's Clothing , Tops , Sets , Suits , Sets</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="J91" t="n">
+        <v>0</v>
+      </c>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t>[['Black-S', 'CJTZ291671201AZ'], ['Black-M', 'CJTZ291671202BY'], ['Black-L', 'CJTZ291671203CX'], ['Black-XL', 'CJTZ291671204DW'], ['Black-2XL', 'CJTZ291671205EV'], ['White-S', 'CJTZ291671206FU'], ['White-M', 'CJTZ291671207GT'], ['White-L', 'CJTZ291671208HS'], ['White-XL', 'CJTZ291671209IR'], ['White-2XL', 'CJTZ291671210JQ']]</t>
+        </is>
+      </c>
+      <c r="L91" t="n">
+        <v>147</v>
+      </c>
+      <c r="M91" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="N91" t="n">
+        <v>1</v>
+      </c>
+      <c r="O91" t="inlineStr"/>
+      <c r="P91" t="inlineStr">
+        <is>
+          <t>CJTZ2916712</t>
+        </is>
+      </c>
+      <c r="Q91" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="R91" t="inlineStr">
+        <is>
+          <t>2061254647762276354</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>m6yayuntu7y30vjvvbrja0ru</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>676716d67602c42f64f06f94</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Collared V-Neck Sleeveless Slit Midi Dress</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>https://cf.cjdropshipping.com/8115ebe0-18dd-469b-97d0-398c79c65b61.png,https://cf.cjdropshipping.com/c8c93881-56c3-408a-8ea2-06f5e5f5adc3.png,https://cf.cjdropshipping.com/65ce6473-c1d4-4587-b63f-ed90cbf25589.png,https://cf.cjdropshipping.com/fc0a10af-b17e-4288-a19c-0e44aa5e6851.png,https://cf.cjdropshipping.com/2b274f63-8f2f-4c4f-b927-11b5ce8a5650.png</t>
+        </is>
+      </c>
+      <c r="E92" t="n">
+        <v>63.4</v>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>Introducing our Collared V-Neck Sleeveless Slit Midi Dress—a perfect blend of sophistication and comfort. This stunning piece features a chic design with a flattering silhouette, ideal for any occasion. The stylish slit adds a touch of allure, ensuring you stand out effortlessly. Dress it up or down for a versatile look!</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>womens</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>Women's Clothing , Tops , Sets , Lady Dresses</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="J92" t="n">
+        <v>2</v>
+      </c>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>[['White-S', 'CJLY291680601AZ'], ['White-M', 'CJLY291680602BY'], ['White-L', 'CJLY291680603CX'], ['White-XL', 'CJLY291680604DW'], ['White-2XL', 'CJLY291680605EV'], ['Dusty Blue-S', 'CJLY291680606FU'], ['Dusty Blue-M', 'CJLY291680607GT'], ['Dusty Blue-L', 'CJLY291680608HS'], ['Dusty Blue-XL', 'CJLY291680609IR'], ['Dusty Blue-2XL', 'CJLY291680610JQ'], ['Charcoal Grey-S', 'CJLY291680611KP'], ['Charcoal Grey-M', 'CJLY291680612LO'], ['Charcoal Grey-L', 'CJLY291680613MN'], ['Charcoal Grey-XL', 'CJLY291680614NM'], ['Charcoal Grey-2XL', 'CJLY291680615OL'], ['Black-S', 'CJLY291680616PK'], ['Black-M', 'CJLY291680617QJ'], ['Black-L', 'CJLY291680618RI'], ['Black-XL', 'CJLY291680619SH'], ['Black-2XL', 'CJLY291680620TG'], ['Lavender Purple-S', 'CJLY291680621UF'], ['Lavender Purple-M', 'CJLY291680622VE'], ['Lavender Purple-L', 'CJLY291680623WD'], ['Lavender Purple-XL', 'CJLY291680624XC'], ['Lavender Purple-2XL', 'CJLY291680625YB']]</t>
+        </is>
+      </c>
+      <c r="L92" t="n">
+        <v>279</v>
+      </c>
+      <c r="M92" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="N92" t="n">
+        <v>1</v>
+      </c>
+      <c r="O92" t="inlineStr"/>
+      <c r="P92" t="inlineStr">
+        <is>
+          <t>CJLY2916806</t>
+        </is>
+      </c>
+      <c r="Q92" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="R92" t="inlineStr">
+        <is>
+          <t>2061274080819957761</t>
         </is>
       </c>
     </row>

</xml_diff>